<commit_message>
BIS-2691: Fixed a typo
</commit_message>
<xml_diff>
--- a/test-integration/sourceTest/resource/IntegrationRoCrateServerTest/metadata_setup.xlsx
+++ b/test-integration/sourceTest/resource/IntegrationRoCrateServerTest/metadata_setup.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="192">
   <si>
     <t xml:space="preserve">VOCABULARY_TYPE</t>
   </si>
@@ -423,9 +423,6 @@
   </si>
   <si>
     <t xml:space="preserve">Children</t>
-  </si>
-  <si>
-    <t xml:space="preserve">openBIS Related Identifiers</t>
   </si>
   <si>
     <t xml:space="preserve">/PUBLICATIONS/PUBLIC_REPOSITORIES/PUB30</t>
@@ -2695,7 +2692,7 @@
         <v>3</v>
       </c>
       <c r="P64" s="2" t="s">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="Q64" s="2" t="s">
         <v>114</v>
@@ -2725,10 +2722,10 @@
         <v>9</v>
       </c>
       <c r="C65" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>118</v>
@@ -2737,43 +2734,43 @@
         <v>123</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K65" s="2"/>
       <c r="L65" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="M65" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="M65" s="2" t="s">
+      <c r="N65" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="N65" s="2" t="s">
+      <c r="O65" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="O65" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="P65" s="2"/>
       <c r="Q65" s="2"/>
       <c r="R65" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="S65" s="2"/>
       <c r="T65" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="U65" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="U65" s="2" t="s">
+      <c r="V65" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="V65" s="2" t="s">
+      <c r="W65" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="W65" s="2" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2782,10 +2779,10 @@
         <v>9</v>
       </c>
       <c r="C66" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>118</v>
@@ -2794,43 +2791,43 @@
         <v>123</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K66" s="2"/>
       <c r="L66" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="M66" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="N66" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="N66" s="2" t="s">
+      <c r="O66" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="O66" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="P66" s="2"/>
       <c r="Q66" s="2"/>
       <c r="R66" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="S66" s="2"/>
       <c r="T66" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="U66" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="U66" s="2" t="s">
+      <c r="V66" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="V66" s="2" t="s">
+      <c r="W66" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="W66" s="2" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2839,10 +2836,10 @@
         <v>9</v>
       </c>
       <c r="C67" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D67" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>118</v>
@@ -2851,43 +2848,43 @@
         <v>123</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K67" s="2"/>
       <c r="L67" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="M67" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N67" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="N67" s="2" t="s">
+      <c r="O67" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="O67" s="2" t="s">
-        <v>162</v>
       </c>
       <c r="P67" s="2"/>
       <c r="Q67" s="2"/>
       <c r="R67" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="S67" s="2"/>
       <c r="T67" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="U67" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="U67" s="2" t="s">
+      <c r="V67" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="W67" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="V67" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="W67" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2956,10 +2953,10 @@
         <v>9</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>118</v>
@@ -2968,15 +2965,15 @@
         <v>123</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="K73" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="K73" s="2" t="s">
-        <v>169</v>
       </c>
       <c r="L73" s="2"/>
       <c r="M73" s="2"/>
@@ -2991,10 +2988,10 @@
         <v>9</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>118</v>
@@ -3003,19 +3000,19 @@
         <v>123</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
       <c r="K74" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="L74" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="L74" s="2" t="s">
+      <c r="M74" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="M74" s="2" t="s">
-        <v>173</v>
       </c>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
@@ -3028,10 +3025,10 @@
         <v>9</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>118</v>
@@ -3040,21 +3037,21 @@
         <v>123</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H75" s="2"/>
       <c r="I75" s="2"/>
       <c r="J75" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="K75" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="K75" s="2" t="s">
+      <c r="L75" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="L75" s="2" t="s">
+      <c r="M75" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="M75" s="2" t="s">
-        <v>178</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -3119,10 +3116,10 @@
         <v>9</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>118</v>
@@ -3131,15 +3128,15 @@
         <v>123</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H81" s="2"/>
       <c r="I81" s="2"/>
       <c r="J81" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="K81" s="2" t="s">
         <v>181</v>
-      </c>
-      <c r="K81" s="2" t="s">
-        <v>182</v>
       </c>
       <c r="L81" s="2"/>
       <c r="M81" s="2"/>
@@ -3150,10 +3147,10 @@
         <v>9</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>118</v>
@@ -3162,27 +3159,27 @@
         <v>123</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H82" s="2"/>
       <c r="I82" s="2"/>
       <c r="J82" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="K82" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="L82" s="2"/>
       <c r="M82" s="2"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3212,16 +3209,16 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>123</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>72</v>
@@ -3230,16 +3227,16 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>123</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>24</v>
@@ -3248,16 +3245,16 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>123</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
BIS-2691: Reverted changes to properties CREATOR and PUBLISHER
</commit_message>
<xml_diff>
--- a/test-integration/sourceTest/resource/IntegrationRoCrateServerTest/metadata_setup.xlsx
+++ b/test-integration/sourceTest/resource/IntegrationRoCrateServerTest/metadata_setup.xlsx
@@ -609,11 +609,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -651,25 +652,6 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Sans"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -731,19 +713,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2436,7 +2418,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
         <v>105</v>
       </c>
@@ -2444,7 +2426,7 @@
         <v>5</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>5</v>
@@ -2485,7 +2467,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
         <v>109</v>
       </c>
@@ -2493,7 +2475,7 @@
         <v>5</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>5</v>
@@ -3279,7 +3261,7 @@
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="atEnd" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
BIS-2737: fixed 'Type Group' into 'Type Groups' column in xls
</commit_message>
<xml_diff>
--- a/test-integration/sourceTest/resource/IntegrationRoCrateServerTest/metadata_setup.xlsx
+++ b/test-integration/sourceTest/resource/IntegrationRoCrateServerTest/metadata_setup.xlsx
@@ -95,7 +95,7 @@
     <t xml:space="preserve">Ontology Version</t>
   </si>
   <si>
-    <t xml:space="preserve">Type Group</t>
+    <t xml:space="preserve">Type Groups</t>
   </si>
   <si>
     <t xml:space="preserve">PERSON</t>
@@ -612,7 +612,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -655,6 +655,13 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -699,7 +706,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -732,6 +739,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1239,7 +1250,7 @@
       <c r="R18" s="5"/>
       <c r="S18" s="5"/>
     </row>
-    <row r="19" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
         <v>1</v>
       </c>
@@ -1267,7 +1278,7 @@
       <c r="I19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="J19" s="8" t="s">
         <v>23</v>
       </c>
       <c r="K19" s="5"/>
@@ -1722,7 +1733,7 @@
       <c r="R33" s="5"/>
       <c r="S33" s="5"/>
     </row>
-    <row r="34" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
         <v>1</v>
       </c>
@@ -1750,7 +1761,7 @@
       <c r="I34" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="J34" s="4" t="s">
+      <c r="J34" s="8" t="s">
         <v>23</v>
       </c>
       <c r="K34" s="5"/>

</xml_diff>